<commit_message>
test: WIP - Add AlleleProfile model converter method to seqdb performance test
</commit_message>
<xml_diff>
--- a/test/seqdb/performance/seq_distance/test_seq_distance_performance.xlsx
+++ b/test/seqdb/performance/seq_distance/test_seq_distance_performance.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\streevdm\gen-epix\gen-epix-api\test\seqdb\performance\seq_distance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B8F99BC9-AA00-4867-9CFE-0CBFAE3D9FE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57876ABE-0BAF-43C2-99D7-9C2B65E224FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15690" yWindow="-15150" windowWidth="21600" windowHeight="11340" activeTab="2" xr2:uid="{7FA6E629-251F-4145-9033-6CE5E058265F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{7FA6E629-251F-4145-9033-6CE5E058265F}"/>
   </bookViews>
   <sheets>
     <sheet name="Organization" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
test: WIP - First implementation of creating demo data for seq distance performance test
</commit_message>
<xml_diff>
--- a/test/seqdb/performance/seq_distance/test_seq_distance_performance.xlsx
+++ b/test/seqdb/performance/seq_distance/test_seq_distance_performance.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\streevdm\gen-epix\gen-epix-api\test\seqdb\performance\seq_distance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57876ABE-0BAF-43C2-99D7-9C2B65E224FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D15DE92-5B66-4DB6-8296-7820B066677E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{7FA6E629-251F-4145-9033-6CE5E058265F}"/>
+    <workbookView xWindow="-27630" yWindow="1170" windowWidth="21600" windowHeight="13890" activeTab="2" xr2:uid="{7FA6E629-251F-4145-9033-6CE5E058265F}"/>
   </bookViews>
   <sheets>
     <sheet name="Organization" sheetId="1" r:id="rId1"/>
@@ -777,16 +777,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A29267CC-6F66-4E20-B1CF-294F0BCE654D}">
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -803,7 +803,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -814,7 +814,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -825,7 +825,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -836,7 +836,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -847,7 +847,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -866,14 +866,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01DA19A5-6033-461B-86DA-76ABA0FF9235}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.28515625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -884,7 +884,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -896,7 +896,7 @@
         <v>dc1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -908,7 +908,7 @@
         <v>dc2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -920,7 +920,7 @@
         <v>dc3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>22</v>
       </c>
@@ -932,7 +932,7 @@
         <v>dc4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -944,7 +944,7 @@
         <v>dc5</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>26</v>
       </c>
@@ -956,7 +956,7 @@
         <v>dc6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>28</v>
       </c>
@@ -968,7 +968,7 @@
         <v>dc7</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>30</v>
       </c>
@@ -980,7 +980,7 @@
         <v>dc8</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>32</v>
       </c>
@@ -992,7 +992,7 @@
         <v>dc9</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>34</v>
       </c>
@@ -1004,7 +1004,7 @@
         <v>dc10</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>36</v>
       </c>
@@ -1024,22 +1024,22 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{385F159A-3559-4F41-A294-33237EBD0730}">
   <dimension ref="A1:M29"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="36.33203125" customWidth="1"/>
-    <col min="3" max="3" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.28515625" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="21" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="36" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.33203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="14.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="25.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="14.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="25.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.7109375" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1080,7 +1080,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>49</v>
       </c>
@@ -1128,7 +1128,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>51</v>
       </c>
@@ -1176,7 +1176,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>53</v>
       </c>
@@ -1224,7 +1224,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>55</v>
       </c>
@@ -1272,7 +1272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>57</v>
       </c>
@@ -1320,7 +1320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>59</v>
       </c>
@@ -1368,7 +1368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>61</v>
       </c>
@@ -1416,7 +1416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>63</v>
       </c>
@@ -1464,7 +1464,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>65</v>
       </c>
@@ -1512,7 +1512,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>67</v>
       </c>
@@ -1560,7 +1560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>69</v>
       </c>
@@ -1608,7 +1608,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>71</v>
       </c>
@@ -1656,7 +1656,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>73</v>
       </c>
@@ -1704,7 +1704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>75</v>
       </c>
@@ -1752,7 +1752,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>77</v>
       </c>
@@ -1800,7 +1800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>79</v>
       </c>
@@ -1848,7 +1848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>81</v>
       </c>
@@ -1896,7 +1896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>83</v>
       </c>
@@ -1944,7 +1944,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>85</v>
       </c>
@@ -1992,7 +1992,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>87</v>
       </c>
@@ -2040,7 +2040,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>89</v>
       </c>
@@ -2088,7 +2088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>91</v>
       </c>
@@ -2136,7 +2136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>93</v>
       </c>
@@ -2184,7 +2184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>95</v>
       </c>
@@ -2232,7 +2232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>97</v>
       </c>
@@ -2280,7 +2280,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>99</v>
       </c>
@@ -2328,7 +2328,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>101</v>
       </c>
@@ -2376,7 +2376,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>103</v>
       </c>

</xml_diff>